<commit_message>
so i just noticed when the program writes the data first time in writes Phone and Mobile as strings. If i delete one of the entries and give them the same dataset it returns me the old data with Phone and Mobile as numbers, the coloring of the cell has been gone(which means probably it overwrites the old data again instead of keeping them intact) and the new entry that i deleted and now got added again is a string. To address the issues im experiencing, u'll make the following changes to the script:
Ensure consistent data types: Keep Phone and Mobile columns as numbers throughout the process.
Avoid overwriting existing data formatting: We will handle the Excel file more carefully to maintain formatting and other properties. Handle each entry seperately , check one by one if its in the xlsx, if not then apend it
</commit_message>
<xml_diff>
--- a/info.xlsx
+++ b/info.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3795" yWindow="3510" windowWidth="24810" windowHeight="11385" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -26,15 +25,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -46,23 +53,33 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Κανονικό" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -425,8 +442,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16.85546875" customWidth="1" min="4" max="4"/>
+    <col width="25.7109375" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -481,28 +502,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2105736150</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>6942632569</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>2105736150</v>
+      </c>
+      <c r="E2" t="n">
+        <v>6942632569</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LAGHIOS ADVANCED DENTISTRY</t>
+          <t>IMS DENTAL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Παπαδιαμαντόπουλου Ιωάννη 4, Ιλίσια, 115 28 Αθήνα Αττικής </t>
+          <t xml:space="preserve">Πλάτωνος 8, Κέντρο, 152 34 Χαλάνδρι Αττικής </t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -510,28 +525,19 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2107213597</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>6944965696</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>2106828072</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>IMS DENTAL</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ABSOLUTE DENTAL CENTER</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Πλάτωνος 8, Κέντρο, 152 34 Χαλάνδρι Αττικής </t>
+          <t xml:space="preserve">Σόλωνος 7, Κολωνάκι, 106 71 Αθήνα Αττικής </t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -539,24 +545,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2106828072</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>2103644903</v>
+      </c>
+      <c r="E4" t="n">
+        <v>6978844744</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABSOLUTE DENTAL CENTER</t>
+          <t>ΕΞΑΡΧΟΥ - ΤΡΙΑΝΤΑΦΥΛΛΟΥ ΝΑΤΑΣΣΑ DENTOLOGY</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Σόλωνος 7, Κολωνάκι, 106 71 Αθήνα Αττικής </t>
+          <t xml:space="preserve">Ελευθερίου Βενιζέλου 72, Ευαγγελίστρια, 146 71 Νέα Ερυθραία Αττικής </t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -564,28 +568,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2103644903</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>6978844744</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>2106200150</v>
+      </c>
+      <c r="E5" t="n">
+        <v>6987525656</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ΕΞΑΡΧΟΥ - ΤΡΙΑΝΤΑΦΥΛΛΟΥ ΝΑΤΑΣΣΑ DENTOLOGY</t>
+          <t>ΜΑΛΛΙΟΥ Ι. ΦΑΝΗ</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ελευθερίου Βενιζέλου 72, Ευαγγελίστρια, 146 71 Νέα Ερυθραία Αττικής </t>
+          <t xml:space="preserve">Λεωφόρος Γαλατσίου 104, 111 46 Γαλάτσι Αττικής </t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -593,28 +591,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2106200150</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>6987525656</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>2102932232</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6977244048</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ΜΑΛΛΙΟΥ Ι. ΦΑΝΗ</t>
+          <t>MEDICAL DENT - ΚΙΜΙΩΝΗΣ ΑΛΕΞΑΝΔΡΟΣ</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Λεωφόρος Γαλατσίου 104, 111 46 Γαλάτσι Αττικής </t>
+          <t xml:space="preserve">Καισαρείας 6, Ιλίσια, 115 27 Αθήνα Αττικής </t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -622,28 +614,19 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2102932232</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>6977244048</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
+      <c r="D7" t="n">
+        <v>2107487200</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MEDICAL DENT - ΚΙΜΙΩΝΗΣ ΑΛΕΞΑΝΔΡΟΣ</t>
+          <t>ΚΥΡΙΑΖΟΣ ΑΛΚΗΣ - YOUR DENTAL CARE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Καισαρείας 6, Ιλίσια, 115 27 Αθήνα Αττικής </t>
+          <t xml:space="preserve">Λεωφόρος Κηφισίας 135 &amp; Λάμψα 1, Αμπελόκηποι, 115 24 Αθήνα Αττικής </t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -651,24 +634,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2107487200</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>2106916337</v>
+      </c>
+      <c r="E8" t="n">
+        <v>6937131148</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ΚΥΡΙΑΖΟΣ ΑΛΚΗΣ - YOUR DENTAL CARE</t>
+          <t>THE DENTAL CLINIC - ΚΑΛΤΣΑΣ ΑΛΕΞΑΝΔΡΟΣ</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Λεωφόρος Κηφισίας 135 &amp; Λάμψα 1, Αμπελόκηποι, 115 24 Αθήνα Αττικής </t>
+          <t xml:space="preserve">Λεωφόρος Κηφισίας 238, Τρίγωνο Αγίας Βαρβάρας, 152 31 Χαλάνδρι Αττικής </t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -676,28 +657,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2106916337</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>6937131148</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>2106745832</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6944293840</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>THE DENTAL CLINIC - ΚΑΛΤΣΑΣ ΑΛΕΞΑΝΔΡΟΣ</t>
+          <t>ΠΟΛΥΟΔΟΝΤΙΑΤΡΕΙΟ DENTAL PLUS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Λεωφόρος Κηφισίας 238, Τρίγωνο Αγίας Βαρβάρας, 152 31 Χαλάνδρι Αττικής </t>
+          <t xml:space="preserve">Λεωφόρος Μαραθώνος 46, 153 51 Παλλήνη Αττικής </t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -705,28 +680,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2106745832</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>6944293840</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>2106669960</v>
+      </c>
+      <c r="E10" t="n">
+        <v>6937605464</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ΠΟΛΥΟΔΟΝΤΙΑΤΡΕΙΟ DENTAL PLUS</t>
+          <t>COSMETIC DENTAL CLINIC</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Λεωφόρος Μαραθώνος 46, 153 51 Παλλήνη Αττικής </t>
+          <t xml:space="preserve">Λεωφόρος Βασιλίσσης Σοφίας 54, Ιλίσια, 115 28 Αθήνα Αττικής </t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -734,28 +703,19 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2106669960</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>6937605464</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>2107296039</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>COSMETIC DENTAL CLINIC</t>
+          <t>ΒΑΤΣΕΛΑ Π. ΕΛΕΝΗ</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Λεωφόρος Βασιλίσσης Σοφίας 54, Ιλίσια, 115 28 Αθήνα Αττικής </t>
+          <t xml:space="preserve">Μελίνας Μερκούρη 20, Άγιοι Ταξιάρχες, 141 22 Ηράκλειο Αττικής </t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -763,24 +723,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2107296039</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>2108216301</v>
+      </c>
+      <c r="E12" t="n">
+        <v>6973787992</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ΒΑΤΣΕΛΑ Π. ΕΛΕΝΗ</t>
+          <t>THE DENTAL HOME</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Μελίνας Μερκούρη 20, Άγιοι Ταξιάρχες, 141 22 Ηράκλειο Αττικής </t>
+          <t xml:space="preserve">Λεωφόρος Περικλέους 27, 155 61 Χολαργός Αττικής </t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -788,28 +746,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2108216301</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>6973787992</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>2106523754</v>
+      </c>
+      <c r="E13" t="n">
+        <v>6972604744</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>THE DENTAL HOME</t>
+          <t>ΛΑΤΙΝΟΣ ΦΩΤΗΣ</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Λεωφόρος Περικλέους 27, 155 61 Χολαργός Αττικής </t>
+          <t xml:space="preserve">Βυζαντινών Αυτοκρατόρων 11, Περισσός, 142 32 Νέα Ιωνία Αττικής </t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -817,28 +769,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2106523754</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>6972604744</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>2102581771</v>
+      </c>
+      <c r="E14" t="n">
+        <v>6974307559</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ΛΑΤΙΝΟΣ ΦΩΤΗΣ</t>
+          <t>ΒΟΓΙΑΤΖΟΓΛΟΥ ΔΗΜΗΤΡΑ</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βυζαντινών Αυτοκρατόρων 11, Περισσός, 142 32 Νέα Ιωνία Αττικής </t>
+          <t xml:space="preserve">Αριστοτέλους 187, 136 78 Αχαρνές Αττικής </t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -846,28 +792,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2102581771</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>6974307559</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>2102464408</v>
+      </c>
+      <c r="E15" t="n">
+        <v>6985689935</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ΒΟΓΙΑΤΖΟΓΛΟΥ ΔΗΜΗΤΡΑ</t>
+          <t>LAGHIOS ADVANCED DENTISTRY</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Αριστοτέλους 187, 136 78 Αχαρνές Αττικής </t>
+          <t xml:space="preserve">Παπαδιαμαντόπουλου Ιωάννη 4, Ιλίσια, 115 28 Αθήνα Αττικής </t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -875,18 +815,12 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>2102464408</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>6985689935</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>2107213597</v>
+      </c>
+      <c r="E16" t="n">
+        <v>6944965696</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -904,28 +838,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>2106439390</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>6943011864</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+      <c r="D17" t="n">
+        <v>2106439390</v>
+      </c>
+      <c r="E17" t="n">
+        <v>6943011864</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ΜΑΡΓΑΡΙΤΗ ΜΑΡΙΑ - DENTAL PROLIPSIS</t>
+          <t>ΚΑΚΛΑΜΑΝΗΣ ΑΓΓΕΛΟΣ - ΠΟΛΥΟΔΟΝΤΙΑΤΡΕΙΟ</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Μπουμπουλίνας 2Α, Αγία Ελεούσα, 176 75 Καλλιθέα Αττικής </t>
+          <t xml:space="preserve">Λεωφόρος Θηβών 210, 121 34 Περιστέρι Αττικής </t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -933,28 +861,19 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>2109583535</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>6976215741</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="D18" t="n">
+        <v>2105730784</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ΚΑΚΛΑΜΑΝΗΣ ΑΓΓΕΛΟΣ - ΠΟΛΥΟΔΟΝΤΙΑΤΡΕΙΟ</t>
+          <t>ΜΑΡΓΑΡΙΤΗ ΜΑΡΙΑ - DENTAL PROLIPSIS</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Λεωφόρος Θηβών 210, 121 34 Περιστέρι Αττικής </t>
+          <t xml:space="preserve">Μπουμπουλίνας 2Α, Αγία Ελεούσα, 176 75 Καλλιθέα Αττικής </t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -962,24 +881,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>2105730784</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="D19" t="n">
+        <v>2109583535</v>
+      </c>
+      <c r="E19" t="n">
+        <v>6976215741</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ΑΝΤΩΝΟΓΙΑΝΝΑΚΗ ΕΥΑΓΓΕΛΙΑ - A-PERIO</t>
+          <t>ΚΑΡΔΑΤΟΥ ΡΟΔΟΠΗ - ΜΑΡΙΑ DMD</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Αναστάσεως 85, Άνω Χολαργός, 155 61 Χολαργός Αττικής </t>
+          <t xml:space="preserve">Λεωφόρος Κύπρου 117, 164 51 Αργυρούπολη Αττικής </t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -987,24 +904,22 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>2106528761</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+      <c r="D20" t="n">
+        <v>2107298955</v>
+      </c>
+      <c r="E20" t="n">
+        <v>6937433366</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ΚΑΡΔΑΤΟΥ ΡΟΔΟΠΗ - ΜΑΡΙΑ DMD</t>
+          <t>ΑΝΤΩΝΟΓΙΑΝΝΑΚΗ ΕΥΑΓΓΕΛΙΑ - A-PERIO</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Λεωφόρος Κύπρου 117, 164 51 Αργυρούπολη Αττικής </t>
+          <t xml:space="preserve">Αναστάσεως 85, Άνω Χολαργός, 155 61 Χολαργός Αττικής </t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1012,68 +927,12 @@
           <t>οδοντιατροι</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>2107298955</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>6937433366</t>
-        </is>
-      </c>
+      <c r="D21" t="n">
+        <v>2106528761</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>ΑΛΕΒΙΖΟΣ ΑΚΗΣ</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Αγίας Φωτεινής 57, Άγιοι Ανάργυροι, 142 31 Νέα Ιωνία Αττικής </t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>οδοντιατροι</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>6972131704</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>ΟΙΚΟΝΟΜΟΥ ΗΛΙΑΣ DDS, MSc - PERIO &amp; ORTHO</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Φειδιππίδου 8, Αμπελόκηποι, 115 26 Αθήνα Αττικής </t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>οδοντιατροι</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>2107770620</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
ready wtf for 1 page but wont close the tabs
</commit_message>
<xml_diff>
--- a/info.xlsx
+++ b/info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\webapp\xo_webscraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7716770-CC05-44A5-A17A-DFD872BCBF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AD894A0-FAE5-4B20-AC3C-3929472C251C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3795" yWindow="3510" windowWidth="24810" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="87">
   <si>
     <t>Name</t>
   </si>
@@ -220,6 +220,60 @@
     <t>6976215741</t>
   </si>
   <si>
+    <t>ΑΝΤΩΝΟΓΙΑΝΝΑΚΗ ΕΥΑΓΓΕΛΙΑ - A-PERIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Αναστάσεως 85, Άνω Χολαργός, 155 61 Χολαργός Αττικής </t>
+  </si>
+  <si>
+    <t>2106528761</t>
+  </si>
+  <si>
+    <t>ΚΑΡΔΑΤΟΥ ΡΟΔΟΠΗ - ΜΑΡΙΑ DMD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Λεωφόρος Κύπρου 117, 164 51 Αργυρούπολη Αττικής </t>
+  </si>
+  <si>
+    <t>2107298955</t>
+  </si>
+  <si>
+    <t>ΑΛΕΒΙΖΟΣ ΑΚΗΣ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Αγίας Φωτεινής 57, Άγιοι Ανάργυροι, 142 31 Νέα Ιωνία Αττικής </t>
+  </si>
+  <si>
+    <t>6972131704</t>
+  </si>
+  <si>
+    <t>ΟΙΚΟΝΟΜΟΥ ΗΛΙΑΣ DDS, MSc - PERIO &amp; ORTHO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Φειδιππίδου 8, Αμπελόκηποι, 115 26 Αθήνα Αττικής </t>
+  </si>
+  <si>
+    <t>2107770620</t>
+  </si>
+  <si>
+    <t>ABSOLUTE DENTAL CENTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Σόλωνος 7, Κολωνάκι, 106 71 Αθήνα Αττικής </t>
+  </si>
+  <si>
+    <t>6978844744</t>
+  </si>
+  <si>
+    <t>MEDICAL DENT - ΚΙΜΙΩΝΗΣ ΑΛΕΞΑΝΔΡΟΣ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Καισαρείας 6, Ιλίσια, 115 27 Αθήνα Αττικής </t>
+  </si>
+  <si>
+    <t>2107487200</t>
+  </si>
+  <si>
     <t>ΚΑΚΛΑΜΑΝΗΣ ΑΓΓΕΛΟΣ - ΠΟΛΥΟΔΟΝΤΙΑΤΡΕΙΟ</t>
   </si>
   <si>
@@ -227,63 +281,6 @@
   </si>
   <si>
     <t>2105730784</t>
-  </si>
-  <si>
-    <t>ΑΝΤΩΝΟΓΙΑΝΝΑΚΗ ΕΥΑΓΓΕΛΙΑ - A-PERIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Αναστάσεως 85, Άνω Χολαργός, 155 61 Χολαργός Αττικής </t>
-  </si>
-  <si>
-    <t>2106528761</t>
-  </si>
-  <si>
-    <t>ΚΑΡΔΑΤΟΥ ΡΟΔΟΠΗ - ΜΑΡΙΑ DMD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Λεωφόρος Κύπρου 117, 164 51 Αργυρούπολη Αττικής </t>
-  </si>
-  <si>
-    <t>2107298955</t>
-  </si>
-  <si>
-    <t>6937433366</t>
-  </si>
-  <si>
-    <t>ΑΛΕΒΙΖΟΣ ΑΚΗΣ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Αγίας Φωτεινής 57, Άγιοι Ανάργυροι, 142 31 Νέα Ιωνία Αττικής </t>
-  </si>
-  <si>
-    <t>6972131704</t>
-  </si>
-  <si>
-    <t>ΟΙΚΟΝΟΜΟΥ ΗΛΙΑΣ DDS, MSc - PERIO &amp; ORTHO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Φειδιππίδου 8, Αμπελόκηποι, 115 26 Αθήνα Αττικής </t>
-  </si>
-  <si>
-    <t>2107770620</t>
-  </si>
-  <si>
-    <t>ABSOLUTE DENTAL CENTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Σόλωνος 7, Κολωνάκι, 106 71 Αθήνα Αττικής </t>
-  </si>
-  <si>
-    <t>2103644903</t>
-  </si>
-  <si>
-    <t>6978844744</t>
-  </si>
-  <si>
-    <t>MEDICAL DENT - ΚΙΜΙΩΝΗΣ ΑΛΕΞΑΝΔΡΟΣ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Καισαρείας 6, Ιλίσια, 115 27 Αθήνα Αττικής </t>
   </si>
 </sst>
 </file>
@@ -658,6 +655,7 @@
   <cols>
     <col min="3" max="3" width="11.5703125" customWidth="1"/>
     <col min="4" max="4" width="14.85546875" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -959,6 +957,9 @@
       <c r="D18" t="s">
         <v>71</v>
       </c>
+      <c r="E18">
+        <v>6937433366</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -973,67 +974,64 @@
       <c r="D19" t="s">
         <v>74</v>
       </c>
-      <c r="E19" t="s">
-        <v>75</v>
-      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" t="s">
         <v>76</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" t="s">
         <v>77</v>
-      </c>
-      <c r="C20" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>78</v>
+      </c>
+      <c r="B21" t="s">
         <v>79</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21">
+        <v>2103644903</v>
+      </c>
+      <c r="E21" t="s">
         <v>80</v>
-      </c>
-      <c r="C21" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" t="s">
         <v>82</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" t="s">
         <v>83</v>
-      </c>
-      <c r="C22" t="s">
-        <v>9</v>
-      </c>
-      <c r="D22" t="s">
-        <v>84</v>
-      </c>
-      <c r="E22" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" t="s">
+        <v>9</v>
+      </c>
+      <c r="D23" t="s">
         <v>86</v>
-      </c>
-      <c r="B23" t="s">
-        <v>87</v>
-      </c>
-      <c r="C23" t="s">
-        <v>9</v>
-      </c>
-      <c r="D23">
-        <v>2107487200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>